<commit_message>
Partners tab: named MNO agreements, subscriber reach, penetration of the 3B partnered base (app + Excel sheet)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ASTS_Valuation_Model.xlsx
+++ b/ASTS_Valuation_Model.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Inputs" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Model" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Stages" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Underwriting" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Partners" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Underwriting" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="315">
   <si>
     <t xml:space="preserve">ASTS Valuation Model — MNO Direct-to-Device Revenue Only</t>
   </si>
@@ -663,6 +664,120 @@
   </si>
   <si>
     <t xml:space="preserve">Stage subs/ARPU/multiples are illustrative editable assumptions from the model owner's framework: growth multiples compress as the story de-risks and growth slows.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARTNERS - ~60 MNO agreements covering 3B+ combined subscribers (AST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Region</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of 3B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agreement / status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vodafone Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Europe / Africa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definitive; SatCo JV for Europe; investor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vodafone Idea (Vi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Announced partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verizon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United States</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definitive commercial agreement; service from 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AT&amp;T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definitive commercial agreement; investor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stc group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saudi / MENA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner; 13 subsidiaries across MENA/Europe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TELUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner (21M total connections)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner; investor (BCE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rakuten Mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founding strategic investor (group: 1.6B members)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named subtotal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All agreements (AST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~60 MNOs; $1.2B+ contracted revenue committed to date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your target penetration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs subscribers / 3B partnered base - the subs input is a penetration assumption on this pool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fleet capacity cross-check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">248 sats x capacity per sat (M subs) - addressable exceeds capacity, so satellites are the bottleneck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subscriber figures are each operator's public totals (approximate, mid-2025/26) - the pool AST can sell into,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not users AST has signed. Rakuten's 1.6B 'members' is its e-commerce ecosystem; the mobile base (~7M) is used here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sources: ast-science.com/partners | Q1 2026 business update (~60 agreements, 3B+ subs, $1.2B+ contracted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">| Via Satellite Oct 2025 (Verizon commercial agreement).</t>
   </si>
   <si>
     <t xml:space="preserve">UNDERWRITING NOTES - what each piece of this model is betting on</t>
@@ -1037,7 +1152,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1167,6 +1282,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3141,6 +3268,270 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="56"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>265</v>
+      </c>
+      <c r="D4" s="33" t="n">
+        <f aca="false">C4/3000</f>
+        <v>0.0883333333333333</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D5" s="33" t="n">
+        <f aca="false">C5/3000</f>
+        <v>0.0666666666666667</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>146</v>
+      </c>
+      <c r="D6" s="33" t="n">
+        <f aca="false">C6/3000</f>
+        <v>0.0486666666666667</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>118</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <f aca="false">C7/3000</f>
+        <v>0.0393333333333333</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <f aca="false">C8/3000</f>
+        <v>0.00833333333333333</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <f aca="false">C9/3000</f>
+        <v>0.00333333333333333</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="33" t="n">
+        <f aca="false">C10/3000</f>
+        <v>0.00333333333333333</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="33" t="n">
+        <f aca="false">C11/3000</f>
+        <v>0.00233333333333333</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C12" s="34" t="n">
+        <f aca="false">SUM(C4:C11)</f>
+        <v>781</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <f aca="false">C12/3000</f>
+        <v>0.260333333333333</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C15" s="35" t="n">
+        <f aca="false">Inputs!$B$5/C13</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="C16" s="24" t="n">
+        <f aca="false">Inputs!$B$15*Inputs!$B$35</f>
+        <v>1984</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:A72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3149,322 +3540,322 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>213</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>215</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>216</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>217</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>218</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>219</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>220</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>221</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>222</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>223</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>224</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>225</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>226</v>
+        <v>264</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>227</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>228</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>229</v>
+        <v>267</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>230</v>
+        <v>268</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>231</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>232</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>233</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>234</v>
+        <v>272</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>235</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>236</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>237</v>
+        <v>275</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>238</v>
+        <v>276</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>239</v>
+        <v>277</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>240</v>
+        <v>278</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>241</v>
+        <v>279</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>242</v>
+        <v>280</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>243</v>
+        <v>281</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>244</v>
+        <v>282</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>245</v>
+        <v>283</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>246</v>
+        <v>284</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>247</v>
+        <v>285</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>248</v>
+        <v>286</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>249</v>
+        <v>287</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>250</v>
+        <v>288</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>251</v>
+        <v>289</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>252</v>
+        <v>290</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>253</v>
+        <v>291</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>254</v>
+        <v>292</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>255</v>
+        <v>293</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>256</v>
+        <v>294</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>257</v>
+        <v>295</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>258</v>
+        <v>296</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>259</v>
+        <v>297</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>260</v>
+        <v>298</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>261</v>
+        <v>299</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>262</v>
+        <v>300</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>263</v>
+        <v>301</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>264</v>
+        <v>302</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>265</v>
+        <v>303</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>266</v>
+        <v>304</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>267</v>
+        <v>305</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>268</v>
+        <v>306</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>269</v>
+        <v>307</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>270</v>
+        <v>308</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>271</v>
+        <v>309</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>272</v>
+        <v>310</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>273</v>
+        <v>311</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>274</v>
+        <v>312</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>275</v>
+        <v>313</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="8" t="s">
-        <v>276</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Label rev/sat ceiling as owner guardrail; add AST's verified revenue-intensity anchors ($150-200M 2026, ~$1B 2027 = ~$10M/sat/yr) and $21-23M Block 2 capex validation
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ASTS_Valuation_Model.xlsx
+++ b/ASTS_Valuation_Model.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="319">
   <si>
     <t xml:space="preserve">ASTS Valuation Model — MNO Direct-to-Device Revenue Only</t>
   </si>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">$M</t>
   </si>
   <si>
-    <t xml:space="preserve">Range $20 - 25M all-in</t>
+    <t xml:space="preserve">AST: avg $21-23M per Block 2 for 90+ units (Q1 2026) - validates this range</t>
   </si>
   <si>
     <t xml:space="preserve">Ground/other D&amp;A at full scale</t>
@@ -273,7 +273,7 @@
     <t xml:space="preserve">$M/sat/yr</t>
   </si>
   <si>
-    <t xml:space="preserve">Flag if a sat must earn more than this per year</t>
+    <t xml:space="preserve">Owner guardrail - AST publishes NO per-sat ceiling; 2027 guidance implies ~$10M/sat/yr (~$1B on 100+ sats)</t>
   </si>
   <si>
     <t xml:space="preserve">Subscriber capacity per sat</t>
@@ -853,6 +853,18 @@
   </si>
   <si>
     <t xml:space="preserve">248 sats: FCC granted constellation authority Apr 2026 (SatNews) - the model's full worldwide build.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue per satellite: NO company ceiling published. Verified anchors (Q1 2026 call): 2026 revenue guidance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$150-200M on ~45 sats by YE26; '~$1B revenue opportunity' in 2027 on 100+ sats = ~$10M/sat/yr guided intensity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The base case asks ~$242M/sat/yr at maturity - ~24x the guided 2027 intensity; the $250M guardrail is the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">model owner's assumption, not AST guidance. AST also states avg Block 2 capex of $21-23M (validates cost input).</t>
   </si>
   <si>
     <t xml:space="preserve">Capacity per satellite: no direct guidance. Published anchors: 10 GHz processing per Block 2 (10x Block 1),</t>
@@ -3532,7 +3544,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A72"/>
+  <dimension ref="A1:A76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="112"/>
@@ -3673,28 +3685,28 @@
         <v>277</v>
       </c>
     </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>278</v>
+      </c>
+    </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
-        <v>278</v>
+      <c r="A32" s="3" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="2" t="s">
         <v>282</v>
       </c>
     </row>
@@ -3703,28 +3715,28 @@
         <v>283</v>
       </c>
     </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>284</v>
+      </c>
+    </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
-        <v>284</v>
+      <c r="A39" s="3" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
         <v>287</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="2" t="s">
         <v>288</v>
       </c>
     </row>
@@ -3738,28 +3750,28 @@
         <v>290</v>
       </c>
     </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>291</v>
+      </c>
+    </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="s">
-        <v>291</v>
+      <c r="A47" s="3" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="2" t="s">
         <v>295</v>
       </c>
     </row>
@@ -3768,28 +3780,28 @@
         <v>296</v>
       </c>
     </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>297</v>
+      </c>
+    </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="2" t="s">
-        <v>297</v>
+      <c r="A54" s="3" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="2" t="s">
         <v>301</v>
       </c>
     </row>
@@ -3808,28 +3820,28 @@
         <v>304</v>
       </c>
     </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
+        <v>305</v>
+      </c>
+    </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="2" t="s">
-        <v>305</v>
+      <c r="A63" s="3" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="3" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
+      <c r="A67" s="2" t="s">
         <v>309</v>
       </c>
     </row>
@@ -3854,8 +3866,28 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="8" t="s">
+      <c r="A72" s="3" t="s">
         <v>314</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="3" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="8" t="s">
+        <v>318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>